<commit_message>
Corrige validación de notebooks, intervalos y prácticas docentes
Separa selección, calibración y prueba; ajusta escaladores dentro de CV,
calibra intervalos temporales sin respuestas futuras y corrige PSI discreto.
Amplía controles de calidad de BoldoNet y precisa el alcance de los datos.

Agrega 28 prácticas con pautas docentes, tiempos coherentes, pasos didácticos,
libro FBA y fuentes M/DAX con controles. Conserva los 13 datos originales.

Validación local: 28 notebooks, 231 celdas, 168 cambios de controles,
10 pruebas metodológicas, 672 enlaces y 36 comprobaciones de pantalla.
</commit_message>
<xml_diff>
--- a/02_Estadistica_Business_Analytics/material_propio/EBA_tablero_excel.xlsx
+++ b/02_Estadistica_Business_Analytics/material_propio/EBA_tablero_excel.xlsx
@@ -15097,77 +15097,77 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Campana</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Tiempo_medio_min</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="B2">
-        <f>COUNTIF(Pedidos!C2:C601,A2)</f>
-        <v/>
-      </c>
-      <c r="C2">
-        <f>AVERAGEIF(Pedidos!C2:C601,A2,Pedidos!E2:E601)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="B3">
-        <f>COUNTIF(Pedidos!C2:C601,A3)</f>
-        <v/>
-      </c>
-      <c r="C3">
-        <f>AVERAGEIF(Pedidos!C2:C601,A3,Pedidos!E2:E601)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="B4">
-        <f>COUNTIF(Pedidos!C2:C601,A4)</f>
-        <v/>
-      </c>
-      <c r="C4">
-        <f>AVERAGEIF(Pedidos!C2:C601,A4,Pedidos!E2:E601)</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
+<s:worksheet xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <s:sheetPr>
+    <s:outlinePr summaryBelow="1" summaryRight="1"/>
+    <s:pageSetUpPr/>
+  </s:sheetPr>
+  <s:dimension ref="A1:C4"/>
+  <s:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <s:sheetData>
+    <s:row r="1">
+      <s:c r="A1" t="inlineStr">
+        <s:is>
+          <s:t>Campana</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B1" t="inlineStr">
+        <s:is>
+          <s:t>n</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="C1" t="inlineStr">
+        <s:is>
+          <s:t>Tiempo_medio_min</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="2">
+      <s:c r="A2" t="inlineStr">
+        <s:is>
+          <s:t>A</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B2">
+        <s:f>COUNTIF(Pedidos!C2:C601,A2)</s:f>
+        <s:v>209.0</s:v>
+      </s:c>
+      <s:c r="C2">
+        <s:f>AVERAGEIF(Pedidos!C2:C601,A2,Pedidos!E2:E601)</s:f>
+        <s:v>40.131196172248806</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="3">
+      <s:c r="A3" t="inlineStr">
+        <s:is>
+          <s:t>B</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B3">
+        <s:f>COUNTIF(Pedidos!C2:C601,A3)</s:f>
+        <s:v>209.0</s:v>
+      </s:c>
+      <s:c r="C3">
+        <s:f>AVERAGEIF(Pedidos!C2:C601,A3,Pedidos!E2:E601)</s:f>
+        <s:v>36.06291866028708</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="4">
+      <s:c r="A4" t="inlineStr">
+        <s:is>
+          <s:t>C</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B4">
+        <s:f>COUNTIF(Pedidos!C2:C601,A4)</s:f>
+        <s:v>182.0</s:v>
+      </s:c>
+      <s:c r="C4">
+        <s:f>AVERAGEIF(Pedidos!C2:C601,A4,Pedidos!E2:E601)</s:f>
+        <s:v>32.028571428571425</s:v>
+      </s:c>
+    </s:row>
+  </s:sheetData>
+  <s:pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</s:worksheet>
 </file>
</xml_diff>